<commit_message>
Enhance executive dashboard functionality and UI
- Implemented character limit handling for questions in the ask endpoint, ensuring valid requests.
- Added new types for executive use case summaries to improve data structure.
- Updated sidebar navigation to reflect accurate counts of insights and actions.
- Modified executive page to improve the display of insights and actions, including better handling of revenue figures.
- Enhanced CSS styles for improved visual clarity and responsiveness in the executive dashboard.
- Updated action center to provide clearer revenue associations and action summaries.
</commit_message>
<xml_diff>
--- a/Context/deal pipeline context/Data Science/Deal Enrichment 29th Sept.xlsx
+++ b/Context/deal pipeline context/Data Science/Deal Enrichment 29th Sept.xlsx
@@ -2,19 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://syrencloud-my.sharepoint.com/personal/tushar_k_syrencloud_com/Documents/Desktop/Projects/NTT Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rabin\OneDrive\Desktop\NTT-Syren\NTT Deal Intelligence\Context\deal pipeline context\Data Science\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{11533BFE-E3C3-4E88-8680-74765DF33338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C23B3453-DA07-4671-B50D-69AA1E42BB3F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE23258A-01A8-4893-805D-E9542C095895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{44CB5419-7BD2-4844-9C12-58EAE615E627}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44CB5419-7BD2-4844-9C12-58EAE615E627}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$2:$N$2</definedName>
+  </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -27,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -821,13 +822,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C571206-F2F1-4BE3-93B8-988D46B1113D}">
   <dimension ref="B2:N22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="7" width="20.5703125" customWidth="1"/>
-    <col min="14" max="14" width="16.5703125" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" customWidth="1"/>
+    <col min="14" max="14" width="16.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -868,7 +870,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>13</v>
       </c>
@@ -900,7 +902,7 @@
         <v>1</v>
       </c>
       <c r="L3">
-        <v>39463</v>
+        <v>5816599</v>
       </c>
       <c r="M3">
         <v>4527</v>
@@ -909,7 +911,7 @@
         <v>38805</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>22</v>
       </c>
@@ -941,7 +943,7 @@
         <v>1</v>
       </c>
       <c r="L4">
-        <v>39463</v>
+        <v>5857719</v>
       </c>
       <c r="M4">
         <v>4527</v>
@@ -950,7 +952,7 @@
         <v>5694</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>28</v>
       </c>
@@ -982,7 +984,7 @@
         <v>1</v>
       </c>
       <c r="L5">
-        <v>31669</v>
+        <v>5767276</v>
       </c>
       <c r="M5">
         <v>5071</v>
@@ -991,7 +993,7 @@
         <v>74043</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>35</v>
       </c>
@@ -1023,7 +1025,7 @@
         <v>1</v>
       </c>
       <c r="L6">
-        <v>24766</v>
+        <v>5692378</v>
       </c>
       <c r="M6">
         <v>3645</v>
@@ -1032,7 +1034,7 @@
         <v>114850</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>42</v>
       </c>
@@ -1064,7 +1066,7 @@
         <v>1</v>
       </c>
       <c r="L7">
-        <v>22230</v>
+        <v>4694876</v>
       </c>
       <c r="M7">
         <v>4331</v>
@@ -1073,7 +1075,7 @@
         <v>6981</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>49</v>
       </c>
@@ -1105,7 +1107,7 @@
         <v>1</v>
       </c>
       <c r="L8">
-        <v>19813</v>
+        <v>5937132</v>
       </c>
       <c r="M8">
         <v>2752</v>
@@ -1114,7 +1116,7 @@
         <v>19985</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>57</v>
       </c>
@@ -1146,7 +1148,7 @@
         <v>1</v>
       </c>
       <c r="L9">
-        <v>19813</v>
+        <v>4017312</v>
       </c>
       <c r="M9">
         <v>2752</v>
@@ -1155,7 +1157,7 @@
         <v>9321</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>62</v>
       </c>
@@ -1187,7 +1189,7 @@
         <v>1</v>
       </c>
       <c r="L10">
-        <v>19813</v>
+        <v>4555960</v>
       </c>
       <c r="M10">
         <v>2752</v>
@@ -1196,7 +1198,7 @@
         <v>8921</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>66</v>
       </c>
@@ -1228,7 +1230,7 @@
         <v>1</v>
       </c>
       <c r="L11">
-        <v>19813</v>
+        <v>4955257</v>
       </c>
       <c r="M11">
         <v>2752</v>
@@ -1237,7 +1239,7 @@
         <v>4124</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>71</v>
       </c>
@@ -1269,7 +1271,7 @@
         <v>1</v>
       </c>
       <c r="L12">
-        <v>19813</v>
+        <v>4399473</v>
       </c>
       <c r="M12">
         <v>2752</v>
@@ -1278,7 +1280,7 @@
         <v>4035</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>75</v>
       </c>
@@ -1310,7 +1312,7 @@
         <v>1</v>
       </c>
       <c r="L13">
-        <v>19813</v>
+        <v>5152334</v>
       </c>
       <c r="M13">
         <v>2752</v>
@@ -1319,7 +1321,7 @@
         <v>1936</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>81</v>
       </c>
@@ -1351,7 +1353,7 @@
         <v>1</v>
       </c>
       <c r="L14">
-        <v>19813</v>
+        <v>4510390</v>
       </c>
       <c r="M14">
         <v>2752</v>
@@ -1360,7 +1362,7 @@
         <v>1788</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>87</v>
       </c>
@@ -1392,7 +1394,7 @@
         <v>1</v>
       </c>
       <c r="L15">
-        <v>19813</v>
+        <v>4210044</v>
       </c>
       <c r="M15">
         <v>2752</v>
@@ -1401,7 +1403,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>92</v>
       </c>
@@ -1433,7 +1435,7 @@
         <v>1</v>
       </c>
       <c r="L16">
-        <v>19813</v>
+        <v>4551280</v>
       </c>
       <c r="M16">
         <v>2752</v>
@@ -1442,7 +1444,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>98</v>
       </c>
@@ -1474,7 +1476,7 @@
         <v>1</v>
       </c>
       <c r="L17">
-        <v>19813</v>
+        <v>5003265</v>
       </c>
       <c r="M17">
         <v>2752</v>
@@ -1483,7 +1485,7 @@
         <v>1425</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>101</v>
       </c>
@@ -1515,7 +1517,7 @@
         <v>1</v>
       </c>
       <c r="L18">
-        <v>19813</v>
+        <v>4225351</v>
       </c>
       <c r="M18">
         <v>2752</v>
@@ -1524,7 +1526,7 @@
         <v>1331</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>105</v>
       </c>
@@ -1556,7 +1558,7 @@
         <v>2</v>
       </c>
       <c r="L19">
-        <v>6573</v>
+        <v>4045362</v>
       </c>
       <c r="M19">
         <v>1176</v>
@@ -1565,7 +1567,7 @@
         <v>142864</v>
       </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>114</v>
       </c>
@@ -1597,7 +1599,7 @@
         <v>2</v>
       </c>
       <c r="L20">
-        <v>6165</v>
+        <v>4926084</v>
       </c>
       <c r="M20">
         <v>1463</v>
@@ -1606,7 +1608,7 @@
         <v>75149</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>121</v>
       </c>
@@ -1638,7 +1640,7 @@
         <v>2</v>
       </c>
       <c r="L21">
-        <v>651</v>
+        <v>5958912</v>
       </c>
       <c r="M21">
         <v>260</v>
@@ -1647,7 +1649,7 @@
         <v>114850</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>124</v>
       </c>
@@ -1679,7 +1681,7 @@
         <v>2</v>
       </c>
       <c r="L22">
-        <v>292</v>
+        <v>4792336</v>
       </c>
       <c r="M22">
         <v>124</v>
@@ -1689,6 +1691,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B2:O2" xr:uid="{8C571206-F2F1-4BE3-93B8-988D46B1113D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: update Deal Enrichment Excel file and refine opportunity details in storyline
</commit_message>
<xml_diff>
--- a/Context/deal pipeline context/Data Science/Deal Enrichment 29th Sept.xlsx
+++ b/Context/deal pipeline context/Data Science/Deal Enrichment 29th Sept.xlsx
@@ -1,24 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rabin\OneDrive\Desktop\NTT-Syren\NTT Deal Intelligence\Context\deal pipeline context\Data Science\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://syrencloud-my.sharepoint.com/personal/tushar_k_syrencloud_com/Documents/Desktop/Projects/NTT Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE23258A-01A8-4893-805D-E9542C095895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{11533BFE-E3C3-4E88-8680-74765DF33338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C23B3453-DA07-4671-B50D-69AA1E42BB3F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44CB5419-7BD2-4844-9C12-58EAE615E627}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{44CB5419-7BD2-4844-9C12-58EAE615E627}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$2:$N$2</definedName>
-  </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,6 +27,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -427,7 +426,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -822,14 +821,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C571206-F2F1-4BE3-93B8-988D46B1113D}">
   <dimension ref="B2:N22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="22.109375" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" customWidth="1"/>
-    <col min="14" max="14" width="16.5546875" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" customWidth="1"/>
+    <col min="14" max="14" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -870,7 +868,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:14">
       <c r="B3" t="s">
         <v>13</v>
       </c>
@@ -902,7 +900,7 @@
         <v>1</v>
       </c>
       <c r="L3">
-        <v>5816599</v>
+        <v>39463</v>
       </c>
       <c r="M3">
         <v>4527</v>
@@ -911,7 +909,7 @@
         <v>38805</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14">
       <c r="B4" t="s">
         <v>22</v>
       </c>
@@ -943,7 +941,7 @@
         <v>1</v>
       </c>
       <c r="L4">
-        <v>5857719</v>
+        <v>39463</v>
       </c>
       <c r="M4">
         <v>4527</v>
@@ -952,7 +950,7 @@
         <v>5694</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:14">
       <c r="B5" t="s">
         <v>28</v>
       </c>
@@ -984,7 +982,7 @@
         <v>1</v>
       </c>
       <c r="L5">
-        <v>5767276</v>
+        <v>31669</v>
       </c>
       <c r="M5">
         <v>5071</v>
@@ -993,7 +991,7 @@
         <v>74043</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:14">
       <c r="B6" t="s">
         <v>35</v>
       </c>
@@ -1025,7 +1023,7 @@
         <v>1</v>
       </c>
       <c r="L6">
-        <v>5692378</v>
+        <v>24766</v>
       </c>
       <c r="M6">
         <v>3645</v>
@@ -1034,7 +1032,7 @@
         <v>114850</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:14">
       <c r="B7" t="s">
         <v>42</v>
       </c>
@@ -1066,7 +1064,7 @@
         <v>1</v>
       </c>
       <c r="L7">
-        <v>4694876</v>
+        <v>22230</v>
       </c>
       <c r="M7">
         <v>4331</v>
@@ -1075,7 +1073,7 @@
         <v>6981</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14">
       <c r="B8" t="s">
         <v>49</v>
       </c>
@@ -1107,7 +1105,7 @@
         <v>1</v>
       </c>
       <c r="L8">
-        <v>5937132</v>
+        <v>19813</v>
       </c>
       <c r="M8">
         <v>2752</v>
@@ -1116,7 +1114,7 @@
         <v>19985</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14">
       <c r="B9" t="s">
         <v>57</v>
       </c>
@@ -1148,7 +1146,7 @@
         <v>1</v>
       </c>
       <c r="L9">
-        <v>4017312</v>
+        <v>19813</v>
       </c>
       <c r="M9">
         <v>2752</v>
@@ -1157,7 +1155,7 @@
         <v>9321</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14">
       <c r="B10" t="s">
         <v>62</v>
       </c>
@@ -1189,7 +1187,7 @@
         <v>1</v>
       </c>
       <c r="L10">
-        <v>4555960</v>
+        <v>19813</v>
       </c>
       <c r="M10">
         <v>2752</v>
@@ -1198,7 +1196,7 @@
         <v>8921</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14">
       <c r="B11" t="s">
         <v>66</v>
       </c>
@@ -1230,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="L11">
-        <v>4955257</v>
+        <v>19813</v>
       </c>
       <c r="M11">
         <v>2752</v>
@@ -1239,7 +1237,7 @@
         <v>4124</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14">
       <c r="B12" t="s">
         <v>71</v>
       </c>
@@ -1271,7 +1269,7 @@
         <v>1</v>
       </c>
       <c r="L12">
-        <v>4399473</v>
+        <v>19813</v>
       </c>
       <c r="M12">
         <v>2752</v>
@@ -1280,7 +1278,7 @@
         <v>4035</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:14">
       <c r="B13" t="s">
         <v>75</v>
       </c>
@@ -1312,7 +1310,7 @@
         <v>1</v>
       </c>
       <c r="L13">
-        <v>5152334</v>
+        <v>19813</v>
       </c>
       <c r="M13">
         <v>2752</v>
@@ -1321,7 +1319,7 @@
         <v>1936</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:14">
       <c r="B14" t="s">
         <v>81</v>
       </c>
@@ -1353,7 +1351,7 @@
         <v>1</v>
       </c>
       <c r="L14">
-        <v>4510390</v>
+        <v>19813</v>
       </c>
       <c r="M14">
         <v>2752</v>
@@ -1362,7 +1360,7 @@
         <v>1788</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:14">
       <c r="B15" t="s">
         <v>87</v>
       </c>
@@ -1394,7 +1392,7 @@
         <v>1</v>
       </c>
       <c r="L15">
-        <v>4210044</v>
+        <v>19813</v>
       </c>
       <c r="M15">
         <v>2752</v>
@@ -1403,7 +1401,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:14">
       <c r="B16" t="s">
         <v>92</v>
       </c>
@@ -1435,7 +1433,7 @@
         <v>1</v>
       </c>
       <c r="L16">
-        <v>4551280</v>
+        <v>19813</v>
       </c>
       <c r="M16">
         <v>2752</v>
@@ -1444,7 +1442,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:14">
       <c r="B17" t="s">
         <v>98</v>
       </c>
@@ -1476,7 +1474,7 @@
         <v>1</v>
       </c>
       <c r="L17">
-        <v>5003265</v>
+        <v>19813</v>
       </c>
       <c r="M17">
         <v>2752</v>
@@ -1485,7 +1483,7 @@
         <v>1425</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:14">
       <c r="B18" t="s">
         <v>101</v>
       </c>
@@ -1517,7 +1515,7 @@
         <v>1</v>
       </c>
       <c r="L18">
-        <v>4225351</v>
+        <v>19813</v>
       </c>
       <c r="M18">
         <v>2752</v>
@@ -1526,7 +1524,7 @@
         <v>1331</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:14">
       <c r="B19" t="s">
         <v>105</v>
       </c>
@@ -1558,7 +1556,7 @@
         <v>2</v>
       </c>
       <c r="L19">
-        <v>4045362</v>
+        <v>6573</v>
       </c>
       <c r="M19">
         <v>1176</v>
@@ -1567,7 +1565,7 @@
         <v>142864</v>
       </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:14">
       <c r="B20" t="s">
         <v>114</v>
       </c>
@@ -1599,7 +1597,7 @@
         <v>2</v>
       </c>
       <c r="L20">
-        <v>4926084</v>
+        <v>6165</v>
       </c>
       <c r="M20">
         <v>1463</v>
@@ -1608,7 +1606,7 @@
         <v>75149</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:14">
       <c r="B21" t="s">
         <v>121</v>
       </c>
@@ -1640,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="L21">
-        <v>5958912</v>
+        <v>651</v>
       </c>
       <c r="M21">
         <v>260</v>
@@ -1649,7 +1647,7 @@
         <v>114850</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:14">
       <c r="B22" t="s">
         <v>124</v>
       </c>
@@ -1681,7 +1679,7 @@
         <v>2</v>
       </c>
       <c r="L22">
-        <v>4792336</v>
+        <v>292</v>
       </c>
       <c r="M22">
         <v>124</v>
@@ -1691,7 +1689,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:O2" xr:uid="{8C571206-F2F1-4BE3-93B8-988D46B1113D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>